<commit_message>
Add Vietnamese SQL module mapping sheet
</commit_message>
<xml_diff>
--- a/permission_matrix.xlsx
+++ b/permission_matrix.xlsx
@@ -8,9 +8,11 @@
   </bookViews>
   <sheets>
     <sheet name="Permission Matrix" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Phân loại SQL" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Permission Matrix'!$A$1:$H$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Phân loại SQL'!$A$1:$C$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,6 +32,11 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="3">
@@ -45,7 +52,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -58,17 +65,28 @@
         <color rgb="00D9DDF4"/>
       </bottom>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00B9BFE5"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -662,4 +680,245 @@
   <autoFilter ref="A1:H5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="105" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Tác dụng</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Module</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="44" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>module1,2.sql</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Script bài tập gốc: tạo lại database, bảng, dữ liệu mẫu, view, procedure và function; có lệnh xóa database nên không chạy trên dữ liệu đang dùng.</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>1 + 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="44" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>01_schema.sql</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Nâng cấp an toàn PhoneStore, bổ sung cột, view, function, procedure và cấu trúc cần cho web; không xóa đơn hàng hiện có.</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="44" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>02_catalog_seed.sql</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Thêm dữ liệu danh mục, thương hiệu và sản phẩm nền ban đầu.</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>03_report_queries.sql</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Các truy vấn báo cáo: sản phẩm đang bán, tồn kho thấp, doanh thu, đơn hàng và khách hàng.</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>04_cleanup_legacy.sql</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Dọn các SKU cũ đã xác định; nếu đã phát sinh giao dịch thì chuyển sang ngừng bán thay vì xóa.</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="44" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>05_product_filters.sql</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Tạo procedure usp_FilterProducts để lọc sản phẩm theo danh mục, thương hiệu và từ khóa.</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="44" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>06_catalog_expand.sql</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Bổ sung catalog mở rộng kèm giá, tồn kho, ảnh, bảo hành và nguồn dữ liệu.</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="44" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>07_checkout.sql</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Tạo procedure usp_CreateOrder, đặt hàng, trừ tồn kho và ghi Orders/OrderItems trong transaction.</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>4 + 5 + 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="44" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>08_demo_accounts.sql</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Tạo tài khoản mẫu admin và user_demo để đăng nhập kiểm thử.</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>2 + 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="44" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>09_check_order_sync.sql</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Kiểm tra web đặt hàng đã đồng bộ dữ liệu vào SQL hay chưa.</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>3 + 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="44" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>14_security_roles.sql</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Tạo role quản trị viên, nhân viên, người xem báo cáo; cấp quyền bằng GRANT và hạn chế bằng DENY.</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="44" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>15_security_tests.sql</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Kiểm thử quyền của từng role, xác nhận thao tác được phép và bị từ chối.</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C13"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>